<commit_message>
updated excel files and excel reader added a new test data provider
</commit_message>
<xml_diff>
--- a/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
+++ b/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
@@ -4,10 +4,10 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="10860" windowHeight="8400"/>
   </bookViews>
   <sheets>
-    <sheet name="Signin page" sheetId="1" r:id="rId1"/>
+    <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -28,24 +28,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="9">
   <si>
-    <t>FieldName</t>
+    <t>UserName</t>
   </si>
   <si>
-    <t>Email</t>
+    <t>Password</t>
   </si>
   <si>
-    <t>Valid_Password</t>
+    <t>ExpectedResults</t>
   </si>
   <si>
-    <t>Invalid_Password</t>
+    <t>scarlevga81@gmail.com</t>
   </si>
   <si>
-    <t>Rule_pssword</t>
+    <t>SZDLMA24j</t>
   </si>
   <si>
-    <t>valid format</t>
+    <t>Valid</t>
+  </si>
+  <si>
+    <t>52664356Trox!!</t>
+  </si>
+  <si>
+    <t>Invalid</t>
+  </si>
+  <si>
+    <t>jamalselowa@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -684,14 +693,20 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1219,35 +1234,72 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="5"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>2</v>
+    <row r="3" spans="1:6">
+      <c r="A3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>3</v>
+    <row r="4" spans="1:6">
+      <c r="A4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>4</v>
+    <row r="5" spans="1:6">
+      <c r="A5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="scarlevga81@gmail.com"/>
+    <hyperlink ref="A3" r:id="rId1" display="scarlevga81@gmail.com"/>
+    <hyperlink ref="A4" r:id="rId2" display="jamalselowa@gmail.com"/>
+    <hyperlink ref="A5" r:id="rId2" display="jamalselowa@gmail.com"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -1256,17 +1308,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1"/>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>5</v>
+      <c r="C1" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test data improved tomorrow we execute the tests for sign in
</commit_message>
<xml_diff>
--- a/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
+++ b/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="10860" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -28,15 +28,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
   <si>
     <t>UserName</t>
   </si>
   <si>
     <t>Password</t>
-  </si>
-  <si>
-    <t>ExpectedResults</t>
   </si>
   <si>
     <t>scarlevga81@gmail.com</t>
@@ -45,13 +42,7 @@
     <t>SZDLMA24j</t>
   </si>
   <si>
-    <t>Valid</t>
-  </si>
-  <si>
     <t>52664356Trox!!</t>
-  </si>
-  <si>
-    <t>Invalid</t>
   </si>
   <si>
     <t>jamalselowa@gmail.com</t>
@@ -1241,56 +1232,43 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>2</v>
-      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" t="s">
-        <v>7</v>
+      <c r="B3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
-      <c r="D4" t="s">
-        <v>4</v>
-      </c>
-      <c r="F4" t="s">
-        <v>7</v>
+      <c r="B4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
-      <c r="D5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" t="s">
-        <v>7</v>
+      <c r="B5" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added new test data provider for invalid login
</commit_message>
<xml_diff>
--- a/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
+++ b/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11520" windowHeight="8400" firstSheet="1" activeTab="2"/>
+    <workbookView windowWidth="13128" windowHeight="8400" firstSheet="1"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
   <si>
     <t>UserName</t>
   </si>
@@ -40,13 +40,13 @@
     <t>scarlevga81@gmail.com</t>
   </si>
   <si>
-    <t>SZDLMA24j</t>
-  </si>
-  <si>
     <t>52664356Trox!!</t>
   </si>
   <si>
     <t>jamalselowa@gmail.com</t>
+  </si>
+  <si>
+    <t>SZDLMA24j</t>
   </si>
   <si>
     <t>Username</t>
@@ -709,7 +709,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -722,7 +722,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1273,35 +1276,29 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
+      <c r="A3" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>4</v>
-      </c>
+      <c r="A5" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="scarlevga81@gmail.com" tooltip="mailto:scarlevga81@gmail.com"/>
-    <hyperlink ref="A3" r:id="rId1" display="scarlevga81@gmail.com"/>
-    <hyperlink ref="A4" r:id="rId2" display="jamalselowa@gmail.com"/>
-    <hyperlink ref="A5" r:id="rId2" display="jamalselowa@gmail.com"/>
+    <hyperlink ref="A3" r:id="rId1" display="jamalselowa@gmail.com" tooltip="mailto:jamalselowa@gmail.com"/>
+    <hyperlink ref="A4" r:id="rId1" display="jamalselowa@gmail.com"/>
+    <hyperlink ref="A2" r:id="rId2" display="scarlevga81@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1377,7 +1374,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Done implementing all tests for sign in
</commit_message>
<xml_diff>
--- a/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
+++ b/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="8400" firstSheet="1"/>
+    <workbookView windowWidth="13128" windowHeight="9000" firstSheet="1" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
   <si>
     <t>UserName</t>
   </si>
@@ -71,6 +71,9 @@
   </si>
   <si>
     <t>26@Mary</t>
+  </si>
+  <si>
+    <t>scarletvega81@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -102,15 +105,15 @@
     <font>
       <u/>
       <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -579,10 +582,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
@@ -716,16 +719,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1257,7 +1260,7 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1268,7 +1271,7 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
@@ -1276,7 +1279,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
@@ -1284,7 +1287,7 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
@@ -1292,7 +1295,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="5"/>
+      <c r="A5" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1326,7 +1329,7 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C2" t="s">
@@ -1337,10 +1340,10 @@
       <c r="A3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1371,7 +1374,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -1379,7 +1382,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="scarlevga81@gmail.com"/>
+    <hyperlink ref="A2" r:id="rId1" display="scarletvega81@gmail.com" tooltip="mailto:scarletvega81@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
new registration data columns added
</commit_message>
<xml_diff>
--- a/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
+++ b/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="9000" firstSheet="1" activeTab="2"/>
+    <workbookView windowWidth="13128" windowHeight="8400" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
   <si>
     <t>UserName</t>
   </si>
@@ -49,31 +49,58 @@
     <t>SZDLMA24j</t>
   </si>
   <si>
-    <t>Username</t>
+    <t>username</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>Jason45</t>
+  </si>
+  <si>
+    <t>test@oddrhymes.com</t>
+  </si>
+  <si>
+    <t>Jamal123</t>
+  </si>
+  <si>
+    <t>test2@outlook</t>
+  </si>
+  <si>
+    <t>Jones50</t>
+  </si>
+  <si>
+    <t>jones12@outlook.com</t>
+  </si>
+  <si>
+    <t>Betty</t>
+  </si>
+  <si>
+    <t>Marriam</t>
+  </si>
+  <si>
+    <t>marriam22@gmail.com</t>
+  </si>
+  <si>
+    <t>Seasonal_Lady!</t>
+  </si>
+  <si>
+    <t>scarletvega81@gmail.com</t>
+  </si>
+  <si>
+    <t>Kamogelo</t>
+  </si>
+  <si>
+    <t>automation@test.com</t>
+  </si>
+  <si>
+    <t>52664356Trox!!!!</t>
   </si>
   <si>
     <t>Email</t>
-  </si>
-  <si>
-    <t>John_Smith</t>
-  </si>
-  <si>
-    <t>john@test.com</t>
-  </si>
-  <si>
-    <t>Test123</t>
-  </si>
-  <si>
-    <t>Marry_Vega</t>
-  </si>
-  <si>
-    <t>mary@@test.com</t>
-  </si>
-  <si>
-    <t>26@Mary</t>
-  </si>
-  <si>
-    <t>scarletvega81@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -712,7 +739,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -721,6 +748,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
@@ -1260,7 +1290,7 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1271,7 +1301,7 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
@@ -1287,7 +1317,7 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
@@ -1311,47 +1341,99 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="3"/>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="28.8" spans="1:4">
+      <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
+      <c r="C1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
+      <c r="C2" s="3">
+        <v>1266</v>
+      </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2">
+        <v>47865</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
         <v>13</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5">
+        <v>48896</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="john@test.com"/>
-    <hyperlink ref="B3" r:id="rId2" display="mary@@test.com"/>
-    <hyperlink ref="C3" r:id="rId3" display="26@Mary"/>
+    <hyperlink ref="B2" r:id="rId1" display="test@oddrhymes.com" tooltip="mailto:test@oddrhymes.com"/>
+    <hyperlink ref="B3" r:id="rId2" display="test2@outlook"/>
+    <hyperlink ref="B6" r:id="rId3" display="marriam22@gmail.com"/>
+    <hyperlink ref="B4" r:id="rId4" display="jones12@outlook.com"/>
+    <hyperlink ref="B7" r:id="rId5" display="scarletvega81@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1366,7 +1448,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1374,7 +1456,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>

</xml_diff>

<commit_message>
registration data provider udate
</commit_message>
<xml_diff>
--- a/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
+++ b/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="8400" activeTab="1"/>
+    <workbookView windowWidth="13128" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
-    <sheet name="Registeration" sheetId="2" r:id="rId2"/>
+    <sheet name="Registration" sheetId="2" r:id="rId2"/>
     <sheet name="ValidLoginCredentials" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>

</xml_diff>

<commit_message>
one test running from the register class
</commit_message>
<xml_diff>
--- a/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
+++ b/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="9000"/>
+    <workbookView windowWidth="13128" windowHeight="9000" firstSheet="1" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Registration" sheetId="2" r:id="rId2"/>
     <sheet name="ValidLoginCredentials" sheetId="3" r:id="rId3"/>
+    <sheet name="RegistrationEmptyEmail" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
   <si>
     <t>UserName</t>
   </si>
@@ -76,31 +77,34 @@
     <t>jones12@outlook.com</t>
   </si>
   <si>
+    <t>marriam</t>
+  </si>
+  <si>
+    <t>marriam22@gmail.com</t>
+  </si>
+  <si>
+    <t>Seasonal_Lady!</t>
+  </si>
+  <si>
+    <t>scarletvega81@gmail.com</t>
+  </si>
+  <si>
+    <t>Kamogelo</t>
+  </si>
+  <si>
+    <t>automation@test.com</t>
+  </si>
+  <si>
+    <t>52664356Trox!!!!</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
     <t>Betty</t>
-  </si>
-  <si>
-    <t>Marriam</t>
-  </si>
-  <si>
-    <t>marriam22@gmail.com</t>
-  </si>
-  <si>
-    <t>Seasonal_Lady!</t>
-  </si>
-  <si>
-    <t>scarletvega81@gmail.com</t>
-  </si>
-  <si>
-    <t>Kamogelo</t>
-  </si>
-  <si>
-    <t>automation@test.com</t>
-  </si>
-  <si>
-    <t>52664356Trox!!!!</t>
-  </si>
-  <si>
-    <t>Email</t>
   </si>
 </sst>
 </file>
@@ -1341,8 +1345,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="3"/>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" ht="28.8" spans="1:4">
       <c r="A1" s="3" t="s">
@@ -1390,50 +1394,42 @@
       <c r="A5" t="s">
         <v>15</v>
       </c>
+      <c r="B5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="C5">
-        <v>48896</v>
+        <v>12345</v>
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" t="s">
-        <v>16</v>
+      <c r="A6" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6">
-        <v>12345</v>
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="4" t="s">
+      <c r="A7" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
+      <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" display="test@oddrhymes.com" tooltip="mailto:test@oddrhymes.com"/>
     <hyperlink ref="B3" r:id="rId2" display="test2@outlook"/>
-    <hyperlink ref="B6" r:id="rId3" display="marriam22@gmail.com"/>
+    <hyperlink ref="B5" r:id="rId3" display="marriam22@gmail.com"/>
     <hyperlink ref="B4" r:id="rId4" display="jones12@outlook.com"/>
-    <hyperlink ref="B7" r:id="rId5" display="scarletvega81@gmail.com"/>
+    <hyperlink ref="B6" r:id="rId5" display="scarletvega81@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1448,7 +1444,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1456,7 +1452,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -1469,4 +1465,36 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2"/>
+      <c r="C2">
+        <v>1266</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
new Registration sheet has been added to check if a weak password can execute with creating a new account methods are to be implemented
</commit_message>
<xml_diff>
--- a/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
+++ b/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="9000" firstSheet="3" activeTab="4"/>
+    <workbookView windowWidth="13128" windowHeight="8400" firstSheet="4" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -12,6 +12,7 @@
     <sheet name="ValidLoginCredentials" sheetId="3" r:id="rId3"/>
     <sheet name="RegistrationEmptyEmail" sheetId="4" r:id="rId4"/>
     <sheet name="EmptyRegisterPassword" sheetId="5" r:id="rId5"/>
+    <sheet name="PasswordWeaknessTest" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
   <si>
     <t>UserName</t>
   </si>
@@ -115,6 +116,15 @@
   </si>
   <si>
     <t>Marriam@test.com</t>
+  </si>
+  <si>
+    <t>Jason12</t>
+  </si>
+  <si>
+    <t>vegajason318</t>
+  </si>
+  <si>
+    <t>abc</t>
   </si>
 </sst>
 </file>
@@ -127,12 +137,21 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -623,156 +642,159 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1304,18 +1326,18 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
@@ -1323,7 +1345,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
@@ -1331,7 +1353,7 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
@@ -1339,7 +1361,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="1"/>
+      <c r="A5" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1359,25 +1381,25 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" ht="28.8" spans="1:4">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="2"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="4">
         <v>1266</v>
       </c>
     </row>
@@ -1385,10 +1407,10 @@
       <c r="A3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>47865</v>
       </c>
     </row>
@@ -1396,7 +1418,7 @@
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1404,7 +1426,7 @@
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>16</v>
       </c>
       <c r="C5">
@@ -1412,10 +1434,10 @@
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C6" t="s">
@@ -1426,10 +1448,10 @@
       <c r="A7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1453,15 +1475,15 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B2" t="s">
@@ -1484,13 +1506,13 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1529,7 +1551,7 @@
       <c r="A2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1540,4 +1562,38 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
All pages implemented and tests updated
</commit_message>
<xml_diff>
--- a/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
+++ b/selenium-framework/src/test/java/com/automation/Resources/Configurations/Test-Data/Test_Data_Fields_Verification.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13128" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9000" firstSheet="2" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -13,6 +13,7 @@
     <sheet name="RegistrationEmptyEmail" sheetId="4" r:id="rId4"/>
     <sheet name="EmptyRegisterPassword" sheetId="5" r:id="rId5"/>
     <sheet name="PasswordWeaknessTest" sheetId="6" r:id="rId6"/>
+    <sheet name="NewUSER" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="31">
   <si>
     <t>UserName</t>
   </si>
@@ -147,6 +148,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
@@ -160,14 +169,6 @@
       <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -645,7 +646,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
@@ -776,22 +777,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyAlignment="1">
@@ -1329,12 +1330,12 @@
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="7" t="s">
@@ -1345,7 +1346,7 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
@@ -1361,7 +1362,7 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="2"/>
+      <c r="A5" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1381,25 +1382,25 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="3"/>
   <sheetData>
     <row r="1" ht="28.8" spans="1:4">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="3"/>
+      <c r="D1" s="2"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="1">
         <v>1266</v>
       </c>
     </row>
@@ -1410,7 +1411,7 @@
       <c r="B3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="4">
         <v>47865</v>
       </c>
     </row>
@@ -1434,7 +1435,7 @@
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="4" t="s">
         <v>17</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -1448,10 +1449,10 @@
       <c r="A7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1475,15 +1476,15 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
       <c r="B2" t="s">
@@ -1506,13 +1507,13 @@
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1551,7 +1552,7 @@
       <c r="A2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1574,7 +1575,7 @@
       <c r="A1" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>22</v>
       </c>
       <c r="C1" t="s">
@@ -1590,6 +1591,40 @@
       </c>
       <c r="C2" t="s">
         <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" ht="28.8" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <v>1266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>